<commit_message>
Update test case reference files. The order of elements in /docProps/app.xml has changed.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/ConditionalFormatting/CFDataBar.xlsx
@@ -396,7 +396,7 @@
       </x:dataBar>
       <x:extLst>
         <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{0cf7a109-a037-492e-9fee-4b588b6e219c}</x14:id>
+          <x14:id>{d93cbe18-200b-4d47-80c5-cb2c911c7530}</x14:id>
         </x:ext>
       </x:extLst>
     </x:cfRule>
@@ -410,7 +410,7 @@
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{0cf7a109-a037-492e-9fee-4b588b6e219c}">
+          <x14:cfRule type="dataBar" id="{d93cbe18-200b-4d47-80c5-cb2c911c7530}">
             <x14:dataBar minLength="0" maxLength="100" showValue="0" gradient="1">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>